<commit_message>
docs: populate version and requirement records from commit changes
</commit_message>
<xml_diff>
--- a/docs/releases/版本紀錄.xlsx
+++ b/docs/releases/版本紀錄.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本控管紀錄" sheetId="1" r:id="Rf4080eca0c1546ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求管理紀錄" sheetId="2" r:id="Re52b2da894b04873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本控管紀錄" sheetId="1" r:id="Rbb6de9f13e444065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求管理紀錄" sheetId="2" r:id="Re16326c596c3450f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,11 +17,175 @@
     <x:comment ref="G5" authorId="0">
       <x:text>
         <x:r>
-          <x:t>來源：https://github.com/peterchen0122/DREAMS1.0/blob/27925065c8c23644ffb5c53c2143fc5b661df336/pyproject.toml#L7
-程式提交：27925065c8c23644ffb5c53c2143fc5b661df336
-原始狀態：待確認發布
+          <x:t>版本來源：https://github.com/peterchen0122/DREAMS1.0/blob/27925065c8c23644ffb5c53c2143fc5b661df336/pyproject.toml#L7
+版本基準：27925065c8c23644ffb5c53c2143fc5b661df336
 原始備註：版本來自專案設定，日期取提交日期；測試清單屬操作規範，不能視為通過紀錄。
-驗證：待補驗證紀錄</x:t>
+原始驗證說明：待補驗證紀錄
+已檢視的功能提交：
+https://github.com/peterchen0122/DREAMS1.0/commit/27925065c8c23644ffb5c53c2143fc5b661df336
+2026-07-28T15:14:40+08:00｜twapd｜no message
+https://github.com/peterchen0122/DREAMS1.0/commit/dbec60465ea1fbbeecb8334ef445d0b81de0e547
+2026-06-22T18:39:36+08:00｜twapd｜no message
+https://github.com/peterchen0122/DREAMS1.0/commit/24f09b6ded597eb3c8d54d11965e4322f5b1fcb2
+2026-05-28T18:54:28+08:00｜twapd｜no message
+https://github.com/peterchen0122/DREAMS1.0/commit/83e7a348db4cda2b7c8fb603618dee8a8c25d6b0
+2026-05-28T18:48:28+08:00｜twapd｜測試驗證
+https://github.com/peterchen0122/DREAMS1.0/commit/35eff9e92c166a3abc2e46bf344753040ded1e2e
+2026-05-28T18:15:37+08:00｜twapd｜Initial DREAMS outstation project
+對應需求：REQ-001、REQ-002、REQ-003、REQ-004、REQ-005</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author/>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="H5" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>依提交的實際程式差異整理；不代表客戶原始提出或已驗收。
+https://github.com/peterchen0122/DREAMS1.0/commit/27925065c8c23644ffb5c53c2143fc5b661df336
+提交日期：2026-07-28T15:14:40+08:00
+作者：twapd
+標題：no message
+異動檔案：
+README.md
+docs/ITRI_DREAMS_TEST_VALIDATION.md
+docs/PV_LOGGER_MQTT_TECH_SPEC.md
+src/dreams_outstation/dnp3_gateway.py
+src/dreams_outstation/service.py
+src/dreams_outstation/state.py
+src/dreams_outstation/web_ui.py
+tests/test_dnp3_gateway.py
+tests/test_dnp3_master_ui.py
+tests/test_service.py
+tests/test_state.py
+tests/test_web_ui.py
+tools/dnp3_master_ui.py</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="H6" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>依提交的實際程式差異整理；不代表客戶原始提出或已驗收。
+https://github.com/peterchen0122/DREAMS1.0/commit/dbec60465ea1fbbeecb8334ef445d0b81de0e547
+提交日期：2026-06-22T18:39:36+08:00
+作者：twapd
+標題：no message
+異動檔案：
+README.md
+config/config.example.yaml
+docs/ITRI_DREAMS_TEST_VALIDATION.md
+docs/PV_LOGGER_MQTT_TECH_SPEC.md
+src/dreams_outstation/config.py
+src/dreams_outstation/dnp3_gateway.py
+src/dreams_outstation/service.py
+src/dreams_outstation/state.py
+src/dreams_outstation/web_ui.py
+tests/test_config.py
+tests/test_dnp3_gateway.py
+tests/test_dnp3_master_ui.py
+tests/test_points.py
+tests/test_service.py
+tests/test_state.py
+tools/dnp3_master_simulator.py
+tools/dnp3_master_ui.py</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="H7" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>依提交的實際程式差異整理；不代表客戶原始提出或已驗收。
+https://github.com/peterchen0122/DREAMS1.0/commit/24f09b6ded597eb3c8d54d11965e4322f5b1fcb2
+提交日期：2026-05-28T18:54:28+08:00
+作者：twapd
+標題：no message
+異動檔案：
+docs/ITRI_DREAMS_TEST_VALIDATION.md
+src/dreams_outstation/service.py
+tests/test_dnp3_master_ui.py
+tests/test_service.py
+tools/dnp3_master_ui.py</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="H8" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>依提交的實際程式差異整理；不代表客戶原始提出或已驗收。
+https://github.com/peterchen0122/DREAMS1.0/commit/83e7a348db4cda2b7c8fb603618dee8a8c25d6b0
+提交日期：2026-05-28T18:48:28+08:00
+作者：twapd
+標題：測試驗證
+異動檔案：
+README.md
+docs/ITRI_DREAMS_TEST_VALIDATION.md
+docs/PV_LOGGER_MQTT_TECH_SPEC.md
+src/dreams_outstation/dnp3_gateway.py
+src/dreams_outstation/service.py
+tests/test_dnp3_master_ui.py
+tests/test_service.py
+tools/dnp3_master_ui.py</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="H9" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>依提交的實際程式差異整理；不代表客戶原始提出或已驗收。
+https://github.com/peterchen0122/DREAMS1.0/commit/35eff9e92c166a3abc2e46bf344753040ded1e2e
+提交日期：2026-05-28T18:15:37+08:00
+作者：twapd
+標題：Initial DREAMS outstation project
+異動檔案：
+.gitignore
+"DREAMS\345\202\263\350\274\270\351\234\200\346\261\202\346\212\200\350\241\223\350\246\217\347\257\204\346\221\230\350\246\201.pdf"
+README.md
+config/config.example.yaml
+deploy/dreams-outstation.service
+docs/PV_LOGGER_MQTT_TECH_SPEC.md
+pyproject.toml
+requirements-dnp3.txt
+requirements.txt
+src/dreams_outstation/__init__.py
+src/dreams_outstation/__main__.py
+src/dreams_outstation/buffer.py
+src/dreams_outstation/command_log.py
+src/dreams_outstation/config.py
+src/dreams_outstation/dnp3_gateway.py
+src/dreams_outstation/dreams_api.py
+src/dreams_outstation/logging_config.py
+src/dreams_outstation/models.py
+src/dreams_outstation/mqtt_client.py
+src/dreams_outstation/points.py
+src/dreams_outstation/service.py
+src/dreams_outstation/site_bindings.py
+src/dreams_outstation/state.py
+src/dreams_outstation/web_ui.py
+tests/test_buffer.py
+tests/test_command_log.py
+tests/test_config.py
+tests/test_dnp3_master_ui.py
+tests/test_dreams_api.py
+tests/test_mqtt_client.py
+tests/test_points.py
+tests/test_service.py
+tests/test_site_bindings.py
+tests/test_state.py
+tests/test_web_ui.py
+tools/dnp3_master_simulator.py
+tools/dnp3_master_ui.py
+"\345\206\215\347\224\237\350\203\275\346\272\220\347\233\243\346\216\247\350\250\255\345\202\231\350\251\246\351\251\227\345\217\212\347\256\241\347\220\206\350\246\217\347\257\204-\345\206\215\347\224\237\350\203\275\346\272\220\347\233\243\346\216\247\350\250\255\345\202\231\351\233\262\347\253\257\350\263\207\346\226\231\347\263\273\347\265\261\350\251\246\351\251\227\345\217\212\347\256\241\347\220\206\350\246\217\347\257\204\345\217\212\345\205\266\345\202\263\350\274\270\351\234\200\346\261\202\346\212\200\350\241\223\350\246\217\347\257\204\346\221\230\350\246\201qa.pdf"
+"\345\206\215\347\224\237\350\203\275\346\272\220\347\233\243\346\216\247\350\250\255\345\202\231\351\233\262\347\253\257\350\263\207\346\226\231\347\263\273\347\265\261\350\251\246\351\251\227\345\217\212\347\256\241\347\220\206\350\246\217\347\257\204.pdf"
+"\345\267\245\347\240\224\351\231\242Dreams\351\233\262\347\253\257\346\270\254\350\251\246\350\246\217\347\257\204\350\252\252\346\230\216_20250918.pdf"</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -75,9 +239,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">總筆數</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">用途：記錄軟體開發與客戶需求的提出、處理與溝通狀況。狀態欄位已設定下拉選單：未開始、進行中、待確認、已完成、已取消。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">需求編號</x:t>
@@ -510,9 +671,9 @@
       </x:c>
       <x:c r="J1" s="9"/>
     </x:row>
-    <x:row r="2" ht="27.149999618530273" customHeight="1">
+    <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>用途：記錄版本異動、發布或修正內容。異動日期依原版本文件或程式提交日期填列；發布未核對者標為「待確認」。</x:v>
+        <x:v>異動內容依程式提交整理，修改人依 commit 作者。發布／驗收未核對者為「待確認」；完整來源見備註附註。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -576,23 +737,28 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="42" customHeight="1">
+    <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="10" t="str">
         <x:v>0.1.0</x:v>
       </x:c>
       <x:c r="B5" s="6" t="n">
         <x:v>46231</x:v>
       </x:c>
-      <x:c r="C5" s="5"/>
+      <x:c r="C5" s="5" t="str">
+        <x:v>REQ-001～
+REQ-005</x:v>
+      </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>專案設定版本為 0.1.0。</x:v>
-      </x:c>
-      <x:c r="E5" s="5"/>
+        <x:v>建立 DNP3／MQTT 點位與 Web 監看；加入多站輪詢、完整快照後啟動及事件時間處理。最新修正保留原始值、離線鎖定、保活與工作失敗判定。</x:v>
+      </x:c>
+      <x:c r="E5" s="5" t="str">
+        <x:v>twapd</x:v>
+      </x:c>
       <x:c r="F5" s="5" t="str">
         <x:v>待確認</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
-        <x:v>程式紀錄，尚無版本標籤；發布待確認。</x:v>
+        <x:v>0.1.0 程式累積紀錄；無發行標籤，發布待確認。</x:v>
       </x:c>
       <x:c r="H5" s="1"/>
       <x:c r="I5" s="3" t="s">
@@ -1835,9 +2001,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64aa8ec7013e4b05"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra911bd59d7b24cb0"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f0bd20269d542fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6728090c0193450c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1875,9 +2041,9 @@
       </x:c>
       <x:c r="K1" s="9"/>
     </x:row>
-    <x:row r="2" ht="27.149999618530273" customHeight="1">
-      <x:c r="A2" s="8" t="s">
-        <x:v>15</x:v>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>需求依已提交程式回填；非原始客戶提出紀錄。提出日期、單位、提出人與期限未提供者留白；驗收待確認。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1914,28 +2080,28 @@
     </x:row>
     <x:row r="4" ht="19.200000762939453" customHeight="1">
       <x:c r="A4" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
+      <x:c r="C4" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="D4" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
+      <x:c r="E4" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="s">
+      <x:c r="F4" s="2" t="s">
         <x:v>20</x:v>
-      </x:c>
-      <x:c r="F4" s="2" t="s">
-        <x:v>21</x:v>
       </x:c>
       <x:c r="G4" s="2" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="H4" s="2" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="3" t="s">
@@ -1946,33 +2112,53 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="16.799999237060547" customHeight="1">
-      <x:c r="A5" s="5"/>
+    <x:row r="5" ht="70" customHeight="1">
+      <x:c r="A5" s="5" t="str">
+        <x:v>REQ-005</x:v>
+      </x:c>
       <x:c r="B5" s="6"/>
       <x:c r="C5" s="5"/>
       <x:c r="D5" s="5"/>
-      <x:c r="E5" s="5"/>
+      <x:c r="E5" s="5" t="str">
+        <x:v>DNP3 原始值保持不變，比例換算只在畫面進行；離線鎖定需明確上線狀態才解除，停用該站 DNP3／週期工作，並修正內部保活與工作失敗判定。</x:v>
+      </x:c>
       <x:c r="F5" s="6"/>
-      <x:c r="G5" s="5"/>
-      <x:c r="H5" s="5"/>
+      <x:c r="G5" s="5" t="str">
+        <x:v>待確認</x:v>
+      </x:c>
+      <x:c r="H5" s="5" t="str">
+        <x:v>依提交回填；2026-07-28
+2792506
+驗收待確認。</x:v>
+      </x:c>
       <x:c r="I5" s="1"/>
       <x:c r="J5" s="3" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="K5" s="4" t="n">
         <x:f>COUNTIF($G$5:$G$104,"待確認")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="16.799999237060547" customHeight="1">
-      <x:c r="A6" s="5"/>
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="5" t="str">
+        <x:v>REQ-004</x:v>
+      </x:c>
       <x:c r="B6" s="6"/>
       <x:c r="C6" s="5"/>
       <x:c r="D6" s="5"/>
-      <x:c r="E6" s="5"/>
+      <x:c r="E6" s="5" t="str">
+        <x:v>調整 AI 事件類別、重啟旗標與主動回報重試；相容多種上線狀態欄位，修正無效 DNP3 時間與模擬器命令回覆。</x:v>
+      </x:c>
       <x:c r="F6" s="6"/>
-      <x:c r="G6" s="5"/>
-      <x:c r="H6" s="5"/>
+      <x:c r="G6" s="5" t="str">
+        <x:v>待確認</x:v>
+      </x:c>
+      <x:c r="H6" s="5" t="str">
+        <x:v>依提交回填；2026-06-22
+dbec604
+驗收待確認。</x:v>
+      </x:c>
       <x:c r="I6" s="1"/>
       <x:c r="J6" s="3" t="s">
         <x:v>12</x:v>
@@ -1982,15 +2168,25 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="16.799999237060547" customHeight="1">
-      <x:c r="A7" s="5"/>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="5" t="str">
+        <x:v>REQ-003</x:v>
+      </x:c>
       <x:c r="B7" s="6"/>
       <x:c r="C7" s="5"/>
       <x:c r="D7" s="5"/>
-      <x:c r="E7" s="5"/>
+      <x:c r="E7" s="5" t="str">
+        <x:v>收到第一份完整快照後才啟動週期工作；事件表新增 DNP3 時間欄位。</x:v>
+      </x:c>
       <x:c r="F7" s="6"/>
-      <x:c r="G7" s="5"/>
-      <x:c r="H7" s="5"/>
+      <x:c r="G7" s="5" t="str">
+        <x:v>待確認</x:v>
+      </x:c>
+      <x:c r="H7" s="5" t="str">
+        <x:v>依提交回填；2026-05-28
+24f09b6
+驗收待確認。</x:v>
+      </x:c>
       <x:c r="I7" s="1"/>
       <x:c r="J7" s="3" t="s">
         <x:v>13</x:v>
@@ -2000,33 +2196,53 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="16.799999237060547" customHeight="1">
-      <x:c r="A8" s="5"/>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="5" t="str">
+        <x:v>REQ-002</x:v>
+      </x:c>
       <x:c r="B8" s="6"/>
       <x:c r="C8" s="5"/>
       <x:c r="D8" s="5"/>
-      <x:c r="E8" s="5"/>
+      <x:c r="E8" s="5" t="str">
+        <x:v>Master 支援多站輪詢／監看及指定單站 AO 操作；依站台離線狀態控制 DNP3 與週期工作。</x:v>
+      </x:c>
       <x:c r="F8" s="6"/>
-      <x:c r="G8" s="5"/>
-      <x:c r="H8" s="5"/>
+      <x:c r="G8" s="5" t="str">
+        <x:v>待確認</x:v>
+      </x:c>
+      <x:c r="H8" s="5" t="str">
+        <x:v>依提交回填；2026-05-28
+83e7a34
+驗收待確認。</x:v>
+      </x:c>
       <x:c r="I8" s="1"/>
       <x:c r="J8" s="3" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="K8" s="4" t="n">
         <x:f>SUM(K3:K7)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="16.799999237060547" customHeight="1">
-      <x:c r="A9" s="5"/>
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="5" t="str">
+        <x:v>REQ-001</x:v>
+      </x:c>
       <x:c r="B9" s="6"/>
       <x:c r="C9" s="5"/>
       <x:c r="D9" s="5"/>
-      <x:c r="E9" s="5"/>
+      <x:c r="E9" s="5" t="str">
+        <x:v>建立 DNP3 Outstation 與 MQTT 閘道，加入點位映射、SQLite 暫存與命令紀錄、站台綁定及 Web 監看／測試介面。</x:v>
+      </x:c>
       <x:c r="F9" s="6"/>
-      <x:c r="G9" s="5"/>
-      <x:c r="H9" s="5"/>
+      <x:c r="G9" s="5" t="str">
+        <x:v>待確認</x:v>
+      </x:c>
+      <x:c r="H9" s="5" t="str">
+        <x:v>依提交回填；2026-05-28
+35eff9e
+驗收待確認。</x:v>
+      </x:c>
       <x:c r="I9" s="1"/>
       <x:c r="J9" s="1"/>
       <x:c r="K9" s="1"/>
@@ -3295,8 +3511,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07fc471ec4ab47d5"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a8605b0bbc14902"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2180db051884e32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>